<commit_message>
add: proptry coverage step definition
</commit_message>
<xml_diff>
--- a/src/data/output/cp_gl_output.xlsx
+++ b/src/data/output/cp_gl_output.xlsx
@@ -1,17 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4459342D-F404-40B0-BF77-8D444F3516C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Output" state="visible" r:id="rId4"/>
+    <sheet name="Output" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Output!$A$1:$I$35</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="133">
   <si>
     <t>Test ID</t>
   </si>
@@ -88,9 +95,6 @@
     <t>TS-013</t>
   </si>
   <si>
-    <t>0099623</t>
-  </si>
-  <si>
     <t>TS-014</t>
   </si>
   <si>
@@ -127,9 +131,6 @@
     <t>TS-022</t>
   </si>
   <si>
-    <t>0099618</t>
-  </si>
-  <si>
     <t>TS-023</t>
   </si>
   <si>
@@ -164,32 +165,284 @@
   </si>
   <si>
     <t>TS-034</t>
+  </si>
+  <si>
+    <t>0099636</t>
+  </si>
+  <si>
+    <t>0099643</t>
+  </si>
+  <si>
+    <t>0099637</t>
+  </si>
+  <si>
+    <t>0099641</t>
+  </si>
+  <si>
+    <t>8867.00</t>
+  </si>
+  <si>
+    <t>575.00</t>
+  </si>
+  <si>
+    <t>212.45</t>
+  </si>
+  <si>
+    <t>9657.70</t>
+  </si>
+  <si>
+    <t>0099638</t>
+  </si>
+  <si>
+    <t>40551.00</t>
+  </si>
+  <si>
+    <t>425.00</t>
+  </si>
+  <si>
+    <t>1216.53</t>
+  </si>
+  <si>
+    <t>42192.53</t>
+  </si>
+  <si>
+    <t>0099644</t>
+  </si>
+  <si>
+    <t>42668.00</t>
+  </si>
+  <si>
+    <t>345.00</t>
+  </si>
+  <si>
+    <t>1280.04</t>
+  </si>
+  <si>
+    <t>44293.04</t>
+  </si>
+  <si>
+    <t>0099639</t>
+  </si>
+  <si>
+    <t>0099646</t>
+  </si>
+  <si>
+    <t>22071.00</t>
+  </si>
+  <si>
+    <t>475.00</t>
+  </si>
+  <si>
+    <t>662.13</t>
+  </si>
+  <si>
+    <t>23208.13</t>
+  </si>
+  <si>
+    <t>0099654</t>
+  </si>
+  <si>
+    <t>47143.00</t>
+  </si>
+  <si>
+    <t>375.00</t>
+  </si>
+  <si>
+    <t>950.36</t>
+  </si>
+  <si>
+    <t>48468.36</t>
+  </si>
+  <si>
+    <t>0099663</t>
+  </si>
+  <si>
+    <t>0099650</t>
+  </si>
+  <si>
+    <t>0099658</t>
+  </si>
+  <si>
+    <t>0099660</t>
+  </si>
+  <si>
+    <t>0099659</t>
+  </si>
+  <si>
+    <t>0099661</t>
+  </si>
+  <si>
+    <t>0099662</t>
+  </si>
+  <si>
+    <t>40378.00</t>
+  </si>
+  <si>
+    <t>325.00</t>
+  </si>
+  <si>
+    <t>814.06</t>
+  </si>
+  <si>
+    <t>41517.06</t>
+  </si>
+  <si>
+    <t>11229.00</t>
+  </si>
+  <si>
+    <t>495.00</t>
+  </si>
+  <si>
+    <t>336.87</t>
+  </si>
+  <si>
+    <t>12060.87</t>
+  </si>
+  <si>
+    <t>28674.50</t>
+  </si>
+  <si>
+    <t>525.00</t>
+  </si>
+  <si>
+    <t>1328.58</t>
+  </si>
+  <si>
+    <t>30528.08</t>
+  </si>
+  <si>
+    <t>0099668</t>
+  </si>
+  <si>
+    <t>18898.00</t>
+  </si>
+  <si>
+    <t>566.94</t>
+  </si>
+  <si>
+    <t>19839.94</t>
+  </si>
+  <si>
+    <t>0099670</t>
+  </si>
+  <si>
+    <t>0099664</t>
+  </si>
+  <si>
+    <t>3367.00</t>
+  </si>
+  <si>
+    <t>385.10</t>
+  </si>
+  <si>
+    <t>168.35</t>
+  </si>
+  <si>
+    <t>3920.45</t>
+  </si>
+  <si>
+    <t>0099669</t>
+  </si>
+  <si>
+    <t>971016.00</t>
+  </si>
+  <si>
+    <t>44202.84</t>
+  </si>
+  <si>
+    <t>1015693.84</t>
+  </si>
+  <si>
+    <t>0099666</t>
+  </si>
+  <si>
+    <t>0099672</t>
+  </si>
+  <si>
+    <t>50107.00</t>
+  </si>
+  <si>
+    <t>1512.96</t>
+  </si>
+  <si>
+    <t>51944.96</t>
+  </si>
+  <si>
+    <t>0099677</t>
+  </si>
+  <si>
+    <t>0099681</t>
+  </si>
+  <si>
+    <t>0099682</t>
+  </si>
+  <si>
+    <t>170994.00</t>
+  </si>
+  <si>
+    <t>5144.07</t>
+  </si>
+  <si>
+    <t>176613.07</t>
+  </si>
+  <si>
+    <t>0099678</t>
+  </si>
+  <si>
+    <t>715907.00</t>
+  </si>
+  <si>
+    <t>545.00</t>
+  </si>
+  <si>
+    <t>21477.21</t>
+  </si>
+  <si>
+    <t>737929.21</t>
+  </si>
+  <si>
+    <t>0099684</t>
+  </si>
+  <si>
+    <t>291863.00</t>
+  </si>
+  <si>
+    <t>225.00</t>
+  </si>
+  <si>
+    <t>8762.64</t>
+  </si>
+  <si>
+    <t>300850.64</t>
+  </si>
+  <si>
+    <t>0099685</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
       <color rgb="FF2C3E50"/>
-      <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -228,7 +481,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -240,6 +493,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -578,23 +832,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I121"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.571428571428571" customWidth="1"/>
-    <col min="2" max="2" width="13.857142857142858" customWidth="1"/>
-    <col min="3" max="3" width="15.142857142857142" customWidth="1"/>
-    <col min="4" max="4" width="13.857142857142858" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="13.571428571428571" customWidth="1"/>
-    <col min="7" max="7" width="18.857142857142858" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="25.428571428571427" customWidth="1"/>
-    <col min="10" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="9" max="9" width="25.44140625" customWidth="1"/>
+    <col min="10" max="24" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -623,431 +877,583 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="5">
         <v>99418</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="5">
         <v>13953</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="5">
         <v>495</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="5">
         <v>418.59</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="5">
         <v>14866.59</v>
       </c>
     </row>
-    <row r="3" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>99497</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="5">
         <v>4642</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="5">
         <v>475</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="5">
         <v>115.14</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="5">
         <v>5233.87</v>
       </c>
     </row>
-    <row r="4" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="3">
-        <v>99508</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>99498</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="5">
         <v>5044</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="5">
         <v>375</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="5">
         <v>121.93</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="5">
         <v>5542.8</v>
       </c>
     </row>
-    <row r="6" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="3">
-        <v>99504</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="3">
-        <v>99499</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+    </row>
+    <row r="8" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="3">
-        <v>99502</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="3">
-        <v>99500</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="3">
-        <v>99505</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="5">
         <v>99506</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="5">
         <v>19501</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="5">
         <v>375</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="5">
         <v>596.28</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="5">
         <v>20472.28</v>
       </c>
     </row>
-    <row r="12" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="5">
         <v>690.96</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="5">
         <v>24117.96</v>
       </c>
     </row>
-    <row r="13" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="3">
-        <v>99514</v>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-    </row>
-    <row r="14" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="10.199999999999999" customHeight="1">
+      <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-    </row>
-    <row r="15" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="B15" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="5">
+        <v>1408.86</v>
+      </c>
+      <c r="F15" s="5">
+        <v>48665.86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="10.199999999999999" customHeight="1">
+      <c r="A16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="3">
-        <v>1408.86</v>
-      </c>
-      <c r="F15" s="3">
-        <v>48665.86</v>
-      </c>
-    </row>
-    <row r="16" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="B16" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="3">
-        <v>99513</v>
-      </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-    </row>
-    <row r="17" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="B17" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="3">
-        <v>99511</v>
-      </c>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-    </row>
-    <row r="18" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-    </row>
-    <row r="19" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="B19" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A20" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="3">
-        <v>99512</v>
-      </c>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-    </row>
-    <row r="20" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="B20" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A21" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-    </row>
-    <row r="21" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="B21" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-    </row>
-    <row r="22" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="B22" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A23" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-    </row>
-    <row r="23" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="B23" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A24" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B24" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A25" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-    </row>
-    <row r="24" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+      <c r="B25" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+    </row>
+    <row r="26" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A26" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-    </row>
-    <row r="25" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+      <c r="B26" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A27" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-    </row>
-    <row r="26" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
+      <c r="B27" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A28" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-    </row>
-    <row r="27" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
+      <c r="B28" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+    </row>
+    <row r="29" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A29" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-    </row>
-    <row r="28" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+      <c r="B29" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A30" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-    </row>
-    <row r="29" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+      <c r="B30" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A31" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-    </row>
-    <row r="30" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
+      <c r="B31" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+    </row>
+    <row r="32" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A32" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-    </row>
-    <row r="31" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
+      <c r="B32" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A33" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-    </row>
-    <row r="32" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
+      <c r="B33" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A34" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-    </row>
-    <row r="33" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="B34" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="10.199999999999999" customHeight="1">
+      <c r="A35" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-    </row>
-    <row r="34" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-    </row>
-    <row r="35" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-    </row>
-    <row r="36" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+    </row>
+    <row r="36" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A36" s="4"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1055,7 +1461,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A37" s="4"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1063,7 +1469,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A38" s="4"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1071,7 +1477,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A39" s="4"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1079,7 +1485,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A40" s="4"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1087,7 +1493,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A41" s="4"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1095,7 +1501,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A42" s="4"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1103,7 +1509,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A43" s="4"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1111,7 +1517,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A44" s="4"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1119,7 +1525,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A45" s="4"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1127,7 +1533,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A46" s="4"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -1135,7 +1541,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A47" s="4"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -1143,7 +1549,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A48" s="4"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -1151,7 +1557,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A49" s="4"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -1159,7 +1565,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A50" s="4"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -1167,7 +1573,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A51" s="4"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -1175,7 +1581,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A52" s="4"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -1183,7 +1589,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A53" s="4"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -1191,7 +1597,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A54" s="4"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -1199,7 +1605,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A55" s="4"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -1207,7 +1613,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A56" s="4"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -1215,7 +1621,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A57" s="4"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -1223,7 +1629,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A58" s="4"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -1231,7 +1637,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A59" s="4"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -1239,7 +1645,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A60" s="4"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -1247,7 +1653,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A61" s="4"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -1255,7 +1661,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A62" s="4"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -1263,7 +1669,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A63" s="4"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -1271,7 +1677,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A64" s="4"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -1279,7 +1685,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A65" s="4"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -1287,7 +1693,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A66" s="4"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -1295,7 +1701,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A67" s="4"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -1303,7 +1709,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A68" s="4"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -1311,7 +1717,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A69" s="4"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -1319,7 +1725,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A70" s="4"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -1327,7 +1733,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A71" s="4"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -1335,7 +1741,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A72" s="4"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -1343,7 +1749,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A73" s="4"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -1351,7 +1757,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A74" s="4"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -1359,7 +1765,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A75" s="4"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -1367,7 +1773,7 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A76" s="4"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -1375,7 +1781,7 @@
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A77" s="4"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -1383,7 +1789,7 @@
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A78" s="4"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -1391,7 +1797,7 @@
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A79" s="4"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -1399,7 +1805,7 @@
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A80" s="4"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -1407,7 +1813,7 @@
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A81" s="4"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -1415,7 +1821,7 @@
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A82" s="4"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -1423,7 +1829,7 @@
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A83" s="4"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -1431,7 +1837,7 @@
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A84" s="4"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -1439,7 +1845,7 @@
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A85" s="4"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -1447,7 +1853,7 @@
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A86" s="4"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -1455,7 +1861,7 @@
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A87" s="4"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -1463,7 +1869,7 @@
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A88" s="4"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -1471,7 +1877,7 @@
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A89" s="4"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -1479,7 +1885,7 @@
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A90" s="4"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -1487,7 +1893,7 @@
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A91" s="4"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -1495,7 +1901,7 @@
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A92" s="4"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -1503,7 +1909,7 @@
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A93" s="4"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -1511,7 +1917,7 @@
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A94" s="4"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -1519,7 +1925,7 @@
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A95" s="4"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -1527,7 +1933,7 @@
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A96" s="4"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -1535,7 +1941,7 @@
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A97" s="4"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -1543,7 +1949,7 @@
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A98" s="4"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -1551,7 +1957,7 @@
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A99" s="4"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -1559,7 +1965,7 @@
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A100" s="4"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -1567,7 +1973,7 @@
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A101" s="4"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -1575,7 +1981,7 @@
       <c r="E101" s="3"/>
       <c r="F101" s="3"/>
     </row>
-    <row r="102" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A102" s="4"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
@@ -1583,7 +1989,7 @@
       <c r="E102" s="3"/>
       <c r="F102" s="3"/>
     </row>
-    <row r="103" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A103" s="4"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -1591,7 +1997,7 @@
       <c r="E103" s="3"/>
       <c r="F103" s="3"/>
     </row>
-    <row r="104" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A104" s="4"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -1599,7 +2005,7 @@
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
     </row>
-    <row r="105" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A105" s="4"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
@@ -1607,7 +2013,7 @@
       <c r="E105" s="3"/>
       <c r="F105" s="3"/>
     </row>
-    <row r="106" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A106" s="4"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
@@ -1615,7 +2021,7 @@
       <c r="E106" s="3"/>
       <c r="F106" s="3"/>
     </row>
-    <row r="107" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A107" s="4"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -1623,7 +2029,7 @@
       <c r="E107" s="3"/>
       <c r="F107" s="3"/>
     </row>
-    <row r="108" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A108" s="4"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
@@ -1631,7 +2037,7 @@
       <c r="E108" s="3"/>
       <c r="F108" s="3"/>
     </row>
-    <row r="109" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A109" s="4"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -1639,7 +2045,7 @@
       <c r="E109" s="3"/>
       <c r="F109" s="3"/>
     </row>
-    <row r="110" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A110" s="4"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -1647,7 +2053,7 @@
       <c r="E110" s="3"/>
       <c r="F110" s="3"/>
     </row>
-    <row r="111" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A111" s="4"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
@@ -1655,7 +2061,7 @@
       <c r="E111" s="3"/>
       <c r="F111" s="3"/>
     </row>
-    <row r="112" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A112" s="4"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -1663,7 +2069,7 @@
       <c r="E112" s="3"/>
       <c r="F112" s="3"/>
     </row>
-    <row r="113" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A113" s="4"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -1671,7 +2077,7 @@
       <c r="E113" s="3"/>
       <c r="F113" s="3"/>
     </row>
-    <row r="114" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A114" s="4"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -1679,7 +2085,7 @@
       <c r="E114" s="3"/>
       <c r="F114" s="3"/>
     </row>
-    <row r="115" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A115" s="4"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -1687,7 +2093,7 @@
       <c r="E115" s="3"/>
       <c r="F115" s="3"/>
     </row>
-    <row r="116" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A116" s="4"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -1695,7 +2101,7 @@
       <c r="E116" s="3"/>
       <c r="F116" s="3"/>
     </row>
-    <row r="117" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A117" s="4"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -1703,7 +2109,7 @@
       <c r="E117" s="3"/>
       <c r="F117" s="3"/>
     </row>
-    <row r="118" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A118" s="4"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -1711,7 +2117,7 @@
       <c r="E118" s="3"/>
       <c r="F118" s="3"/>
     </row>
-    <row r="119" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A119" s="4"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -1719,7 +2125,7 @@
       <c r="E119" s="3"/>
       <c r="F119" s="3"/>
     </row>
-    <row r="120" ht="12.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A120" s="4"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -1727,11 +2133,11 @@
       <c r="E120" s="3"/>
       <c r="F120" s="3"/>
     </row>
-    <row r="121" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A121" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: various fixes and code and data
</commit_message>
<xml_diff>
--- a/src/data/output/cp_gl_output.xlsx
+++ b/src/data/output/cp_gl_output.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4459342D-F404-40B0-BF77-8D444F3516C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C09FC43-0AAC-47CB-B7B5-762E91597FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -446,12 +446,24 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -481,7 +493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -493,7 +505,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -881,19 +898,19 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="3">
         <v>99418</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="3">
         <v>13953</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="3">
         <v>495</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="3">
         <v>418.59</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="3">
         <v>14866.59</v>
       </c>
     </row>
@@ -901,51 +918,51 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="3">
         <v>99497</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3">
         <v>4642</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="3">
         <v>475</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="3">
         <v>115.14</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="3">
         <v>5233.87</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="10.199999999999999" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>99498</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <v>5044</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="3">
         <v>375</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="3">
         <v>121.93</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="3">
         <v>5542.8</v>
       </c>
     </row>
@@ -953,43 +970,43 @@
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="3" t="s">
         <v>56</v>
       </c>
     </row>
@@ -997,19 +1014,19 @@
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="3" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1017,19 +1034,19 @@
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="3" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1037,19 +1054,19 @@
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="3">
         <v>99506</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="3">
         <v>19501</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="3">
         <v>375</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="3">
         <v>596.28</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="3">
         <v>20472.28</v>
       </c>
     </row>
@@ -1057,19 +1074,19 @@
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="3">
         <v>690.96</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="3">
         <v>24117.96</v>
       </c>
     </row>
@@ -1077,31 +1094,31 @@
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:9" ht="10.199999999999999" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="3" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1109,19 +1126,19 @@
       <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="3">
         <v>1408.86</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="3">
         <v>48665.86</v>
       </c>
     </row>
@@ -1129,19 +1146,19 @@
       <c r="A16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="3" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1149,19 +1166,19 @@
       <c r="A17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1169,235 +1186,235 @@
       <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="3" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="3" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
     </row>
     <row r="24" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="3" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="3" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E27" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" s="3" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
     </row>
     <row r="29" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" s="3" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="10.199999999999999" customHeight="1">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
     </row>
     <row r="31" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
     </row>
     <row r="32" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E32" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F32" s="3" t="s">
         <v>121</v>
       </c>
     </row>
@@ -1405,19 +1422,19 @@
       <c r="A33" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E33" s="5" t="s">
+      <c r="E33" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="F33" s="5" t="s">
+      <c r="F33" s="3" t="s">
         <v>126</v>
       </c>
     </row>
@@ -1425,19 +1442,19 @@
       <c r="A34" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E34" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="3" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1445,13 +1462,13 @@
       <c r="A35" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
     </row>
     <row r="36" spans="1:6" ht="10.199999999999999" customHeight="1">
       <c r="A36" s="4"/>

</xml_diff>